<commit_message>
Support nullable emails and role-column assignment in employee import
Employee import no longer requires an email (generates none if missing),
honors a Role/Access Level column to set or preserve member roles instead
of always defaulting to EMPLOYEE, and updates dependent employee/profile/
notification/dwms-directory lookups to handle a nullable email.
</commit_message>
<xml_diff>
--- a/Gemba_EMS_Employee_Onboarding_Template.xlsx
+++ b/Gemba_EMS_Employee_Onboarding_Template.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:C18"/>
+  <dimension ref="B1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -569,7 +569,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>At least one contact is recommended. If omitted, a placeholder is generated.</t>
+          <t>At least one contact is recommended, but not required — left blank if unknown.</t>
         </is>
       </c>
     </row>
@@ -669,37 +669,49 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
+    <row r="15" ht="60" customHeight="1">
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Re-import:</t>
+          <t>Access Level:</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Safe to re-upload — existing employees matched by Employee Code are updated, not duplicated.</t>
+          <t>Administrator | Management | Human Resources | Head of Department | Employee. Sets the person's system role and always applies when filled in — even on re-import, overriding a role changed in Settings &gt; Members. Leave blank on re-import to keep an existing member's current role; defaults new employees to Employee.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
         <is>
+          <t>Re-import:</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Safe to re-upload — existing employees matched by Employee Code are updated, not duplicated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="2" t="inlineStr">
+        <is>
           <t>Dry run:</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Use the 'Test Import' button first to preview results without saving.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="B18" s="2" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>EXAMPLE row:</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>The yellow row in 'Employee Data' is for reference only — it is automatically skipped.</t>
         </is>
@@ -719,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U203"/>
+  <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -740,9 +752,10 @@
     <col width="26" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="26" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -761,7 +774,7 @@
           <t>WORK ALLOCATION</t>
         </is>
       </c>
-      <c r="S1" s="5" t="inlineStr">
+      <c r="T1" s="5" t="inlineStr">
         <is>
           <t>ROLE &amp; SKILLS</t>
         </is>
@@ -878,17 +891,23 @@
       </c>
       <c r="S2" s="6" t="inlineStr">
         <is>
+          <t>Access Level
+System role — see Instructions tab</t>
+        </is>
+      </c>
+      <c r="T2" s="6" t="inlineStr">
+        <is>
           <t>Primary Work Role
 Main function / job description</t>
         </is>
       </c>
-      <c r="T2" s="6" t="inlineStr">
+      <c r="U2" s="6" t="inlineStr">
         <is>
           <t>Skill Level
 Beginner / Intermediate / Advanced</t>
         </is>
       </c>
-      <c r="U2" s="6" t="inlineStr">
+      <c r="V2" s="6" t="inlineStr">
         <is>
           <t>Training Needed
 Yes / No</t>
@@ -988,15 +1007,20 @@
       </c>
       <c r="S3" s="8" t="inlineStr">
         <is>
+          <t>Employee</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
           <t>Machine Operator</t>
         </is>
       </c>
-      <c r="T3" s="8" t="inlineStr">
+      <c r="U3" s="8" t="inlineStr">
         <is>
           <t>Intermediate</t>
         </is>
       </c>
-      <c r="U3" s="8" t="inlineStr">
+      <c r="V3" s="8" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -1026,6 +1050,7 @@
       <c r="S4" s="10" t="n"/>
       <c r="T4" s="10" t="n"/>
       <c r="U4" s="10" t="n"/>
+      <c r="V4" s="10" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="9" t="n">
@@ -1051,6 +1076,7 @@
       <c r="S5" s="10" t="n"/>
       <c r="T5" s="10" t="n"/>
       <c r="U5" s="10" t="n"/>
+      <c r="V5" s="10" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="9" t="n">
@@ -1076,6 +1102,7 @@
       <c r="S6" s="10" t="n"/>
       <c r="T6" s="10" t="n"/>
       <c r="U6" s="10" t="n"/>
+      <c r="V6" s="10" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="9" t="n">
@@ -1101,6 +1128,7 @@
       <c r="S7" s="10" t="n"/>
       <c r="T7" s="10" t="n"/>
       <c r="U7" s="10" t="n"/>
+      <c r="V7" s="10" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="9" t="n">
@@ -1126,6 +1154,7 @@
       <c r="S8" s="10" t="n"/>
       <c r="T8" s="10" t="n"/>
       <c r="U8" s="10" t="n"/>
+      <c r="V8" s="10" t="n"/>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="9" t="n">
@@ -1151,6 +1180,7 @@
       <c r="S9" s="10" t="n"/>
       <c r="T9" s="10" t="n"/>
       <c r="U9" s="10" t="n"/>
+      <c r="V9" s="10" t="n"/>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="9" t="n">
@@ -1176,6 +1206,7 @@
       <c r="S10" s="10" t="n"/>
       <c r="T10" s="10" t="n"/>
       <c r="U10" s="10" t="n"/>
+      <c r="V10" s="10" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="9" t="n">
@@ -1201,6 +1232,7 @@
       <c r="S11" s="10" t="n"/>
       <c r="T11" s="10" t="n"/>
       <c r="U11" s="10" t="n"/>
+      <c r="V11" s="10" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="9" t="n">
@@ -1226,6 +1258,7 @@
       <c r="S12" s="10" t="n"/>
       <c r="T12" s="10" t="n"/>
       <c r="U12" s="10" t="n"/>
+      <c r="V12" s="10" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="9" t="n">
@@ -1251,6 +1284,7 @@
       <c r="S13" s="10" t="n"/>
       <c r="T13" s="10" t="n"/>
       <c r="U13" s="10" t="n"/>
+      <c r="V13" s="10" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="9" t="n">
@@ -1276,6 +1310,7 @@
       <c r="S14" s="10" t="n"/>
       <c r="T14" s="10" t="n"/>
       <c r="U14" s="10" t="n"/>
+      <c r="V14" s="10" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="9" t="n">
@@ -1301,6 +1336,7 @@
       <c r="S15" s="10" t="n"/>
       <c r="T15" s="10" t="n"/>
       <c r="U15" s="10" t="n"/>
+      <c r="V15" s="10" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="9" t="n">
@@ -1326,6 +1362,7 @@
       <c r="S16" s="10" t="n"/>
       <c r="T16" s="10" t="n"/>
       <c r="U16" s="10" t="n"/>
+      <c r="V16" s="10" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="9" t="n">
@@ -1351,6 +1388,7 @@
       <c r="S17" s="10" t="n"/>
       <c r="T17" s="10" t="n"/>
       <c r="U17" s="10" t="n"/>
+      <c r="V17" s="10" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="9" t="n">
@@ -1376,6 +1414,7 @@
       <c r="S18" s="10" t="n"/>
       <c r="T18" s="10" t="n"/>
       <c r="U18" s="10" t="n"/>
+      <c r="V18" s="10" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="9" t="n">
@@ -1401,6 +1440,7 @@
       <c r="S19" s="10" t="n"/>
       <c r="T19" s="10" t="n"/>
       <c r="U19" s="10" t="n"/>
+      <c r="V19" s="10" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="9" t="n">
@@ -1426,6 +1466,7 @@
       <c r="S20" s="10" t="n"/>
       <c r="T20" s="10" t="n"/>
       <c r="U20" s="10" t="n"/>
+      <c r="V20" s="10" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="9" t="n">
@@ -1451,6 +1492,7 @@
       <c r="S21" s="10" t="n"/>
       <c r="T21" s="10" t="n"/>
       <c r="U21" s="10" t="n"/>
+      <c r="V21" s="10" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="9" t="n">
@@ -1476,6 +1518,7 @@
       <c r="S22" s="10" t="n"/>
       <c r="T22" s="10" t="n"/>
       <c r="U22" s="10" t="n"/>
+      <c r="V22" s="10" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="9" t="n">
@@ -1501,6 +1544,7 @@
       <c r="S23" s="10" t="n"/>
       <c r="T23" s="10" t="n"/>
       <c r="U23" s="10" t="n"/>
+      <c r="V23" s="10" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="9" t="n">
@@ -1526,6 +1570,7 @@
       <c r="S24" s="10" t="n"/>
       <c r="T24" s="10" t="n"/>
       <c r="U24" s="10" t="n"/>
+      <c r="V24" s="10" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="9" t="n">
@@ -1551,6 +1596,7 @@
       <c r="S25" s="10" t="n"/>
       <c r="T25" s="10" t="n"/>
       <c r="U25" s="10" t="n"/>
+      <c r="V25" s="10" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="9" t="n">
@@ -1576,6 +1622,7 @@
       <c r="S26" s="10" t="n"/>
       <c r="T26" s="10" t="n"/>
       <c r="U26" s="10" t="n"/>
+      <c r="V26" s="10" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="9" t="n">
@@ -1601,6 +1648,7 @@
       <c r="S27" s="10" t="n"/>
       <c r="T27" s="10" t="n"/>
       <c r="U27" s="10" t="n"/>
+      <c r="V27" s="10" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="9" t="n">
@@ -1626,6 +1674,7 @@
       <c r="S28" s="10" t="n"/>
       <c r="T28" s="10" t="n"/>
       <c r="U28" s="10" t="n"/>
+      <c r="V28" s="10" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="9" t="n">
@@ -1651,6 +1700,7 @@
       <c r="S29" s="10" t="n"/>
       <c r="T29" s="10" t="n"/>
       <c r="U29" s="10" t="n"/>
+      <c r="V29" s="10" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="9" t="n">
@@ -1676,6 +1726,7 @@
       <c r="S30" s="10" t="n"/>
       <c r="T30" s="10" t="n"/>
       <c r="U30" s="10" t="n"/>
+      <c r="V30" s="10" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="9" t="n">
@@ -1701,6 +1752,7 @@
       <c r="S31" s="10" t="n"/>
       <c r="T31" s="10" t="n"/>
       <c r="U31" s="10" t="n"/>
+      <c r="V31" s="10" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="9" t="n">
@@ -1726,6 +1778,7 @@
       <c r="S32" s="10" t="n"/>
       <c r="T32" s="10" t="n"/>
       <c r="U32" s="10" t="n"/>
+      <c r="V32" s="10" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="9" t="n">
@@ -1751,6 +1804,7 @@
       <c r="S33" s="10" t="n"/>
       <c r="T33" s="10" t="n"/>
       <c r="U33" s="10" t="n"/>
+      <c r="V33" s="10" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="9" t="n">
@@ -1776,6 +1830,7 @@
       <c r="S34" s="10" t="n"/>
       <c r="T34" s="10" t="n"/>
       <c r="U34" s="10" t="n"/>
+      <c r="V34" s="10" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="9" t="n">
@@ -1801,6 +1856,7 @@
       <c r="S35" s="10" t="n"/>
       <c r="T35" s="10" t="n"/>
       <c r="U35" s="10" t="n"/>
+      <c r="V35" s="10" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="9" t="n">
@@ -1826,6 +1882,7 @@
       <c r="S36" s="10" t="n"/>
       <c r="T36" s="10" t="n"/>
       <c r="U36" s="10" t="n"/>
+      <c r="V36" s="10" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="9" t="n">
@@ -1851,6 +1908,7 @@
       <c r="S37" s="10" t="n"/>
       <c r="T37" s="10" t="n"/>
       <c r="U37" s="10" t="n"/>
+      <c r="V37" s="10" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="9" t="n">
@@ -1876,6 +1934,7 @@
       <c r="S38" s="10" t="n"/>
       <c r="T38" s="10" t="n"/>
       <c r="U38" s="10" t="n"/>
+      <c r="V38" s="10" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="9" t="n">
@@ -1901,6 +1960,7 @@
       <c r="S39" s="10" t="n"/>
       <c r="T39" s="10" t="n"/>
       <c r="U39" s="10" t="n"/>
+      <c r="V39" s="10" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="9" t="n">
@@ -1926,6 +1986,7 @@
       <c r="S40" s="10" t="n"/>
       <c r="T40" s="10" t="n"/>
       <c r="U40" s="10" t="n"/>
+      <c r="V40" s="10" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="9" t="n">
@@ -1951,6 +2012,7 @@
       <c r="S41" s="10" t="n"/>
       <c r="T41" s="10" t="n"/>
       <c r="U41" s="10" t="n"/>
+      <c r="V41" s="10" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="9" t="n">
@@ -1976,6 +2038,7 @@
       <c r="S42" s="10" t="n"/>
       <c r="T42" s="10" t="n"/>
       <c r="U42" s="10" t="n"/>
+      <c r="V42" s="10" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="9" t="n">
@@ -2001,6 +2064,7 @@
       <c r="S43" s="10" t="n"/>
       <c r="T43" s="10" t="n"/>
       <c r="U43" s="10" t="n"/>
+      <c r="V43" s="10" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="9" t="n">
@@ -2026,6 +2090,7 @@
       <c r="S44" s="10" t="n"/>
       <c r="T44" s="10" t="n"/>
       <c r="U44" s="10" t="n"/>
+      <c r="V44" s="10" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="9" t="n">
@@ -2051,6 +2116,7 @@
       <c r="S45" s="10" t="n"/>
       <c r="T45" s="10" t="n"/>
       <c r="U45" s="10" t="n"/>
+      <c r="V45" s="10" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="9" t="n">
@@ -2076,6 +2142,7 @@
       <c r="S46" s="10" t="n"/>
       <c r="T46" s="10" t="n"/>
       <c r="U46" s="10" t="n"/>
+      <c r="V46" s="10" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="9" t="n">
@@ -2101,6 +2168,7 @@
       <c r="S47" s="10" t="n"/>
       <c r="T47" s="10" t="n"/>
       <c r="U47" s="10" t="n"/>
+      <c r="V47" s="10" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="9" t="n">
@@ -2126,6 +2194,7 @@
       <c r="S48" s="10" t="n"/>
       <c r="T48" s="10" t="n"/>
       <c r="U48" s="10" t="n"/>
+      <c r="V48" s="10" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="9" t="n">
@@ -2151,6 +2220,7 @@
       <c r="S49" s="10" t="n"/>
       <c r="T49" s="10" t="n"/>
       <c r="U49" s="10" t="n"/>
+      <c r="V49" s="10" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="9" t="n">
@@ -2176,6 +2246,7 @@
       <c r="S50" s="10" t="n"/>
       <c r="T50" s="10" t="n"/>
       <c r="U50" s="10" t="n"/>
+      <c r="V50" s="10" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="9" t="n">
@@ -2201,6 +2272,7 @@
       <c r="S51" s="10" t="n"/>
       <c r="T51" s="10" t="n"/>
       <c r="U51" s="10" t="n"/>
+      <c r="V51" s="10" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="9" t="n">
@@ -2226,6 +2298,7 @@
       <c r="S52" s="10" t="n"/>
       <c r="T52" s="10" t="n"/>
       <c r="U52" s="10" t="n"/>
+      <c r="V52" s="10" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="9" t="n">
@@ -2251,6 +2324,7 @@
       <c r="S53" s="10" t="n"/>
       <c r="T53" s="10" t="n"/>
       <c r="U53" s="10" t="n"/>
+      <c r="V53" s="10" t="n"/>
     </row>
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="9" t="n">
@@ -2276,6 +2350,7 @@
       <c r="S54" s="10" t="n"/>
       <c r="T54" s="10" t="n"/>
       <c r="U54" s="10" t="n"/>
+      <c r="V54" s="10" t="n"/>
     </row>
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="9" t="n">
@@ -2301,6 +2376,7 @@
       <c r="S55" s="10" t="n"/>
       <c r="T55" s="10" t="n"/>
       <c r="U55" s="10" t="n"/>
+      <c r="V55" s="10" t="n"/>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="9" t="n">
@@ -2326,6 +2402,7 @@
       <c r="S56" s="10" t="n"/>
       <c r="T56" s="10" t="n"/>
       <c r="U56" s="10" t="n"/>
+      <c r="V56" s="10" t="n"/>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="9" t="n">
@@ -2351,6 +2428,7 @@
       <c r="S57" s="10" t="n"/>
       <c r="T57" s="10" t="n"/>
       <c r="U57" s="10" t="n"/>
+      <c r="V57" s="10" t="n"/>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="9" t="n">
@@ -2376,6 +2454,7 @@
       <c r="S58" s="10" t="n"/>
       <c r="T58" s="10" t="n"/>
       <c r="U58" s="10" t="n"/>
+      <c r="V58" s="10" t="n"/>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="9" t="n">
@@ -2401,6 +2480,7 @@
       <c r="S59" s="10" t="n"/>
       <c r="T59" s="10" t="n"/>
       <c r="U59" s="10" t="n"/>
+      <c r="V59" s="10" t="n"/>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="9" t="n">
@@ -2426,6 +2506,7 @@
       <c r="S60" s="10" t="n"/>
       <c r="T60" s="10" t="n"/>
       <c r="U60" s="10" t="n"/>
+      <c r="V60" s="10" t="n"/>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="9" t="n">
@@ -2451,6 +2532,7 @@
       <c r="S61" s="10" t="n"/>
       <c r="T61" s="10" t="n"/>
       <c r="U61" s="10" t="n"/>
+      <c r="V61" s="10" t="n"/>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="9" t="n">
@@ -2476,6 +2558,7 @@
       <c r="S62" s="10" t="n"/>
       <c r="T62" s="10" t="n"/>
       <c r="U62" s="10" t="n"/>
+      <c r="V62" s="10" t="n"/>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="9" t="n">
@@ -2501,6 +2584,7 @@
       <c r="S63" s="10" t="n"/>
       <c r="T63" s="10" t="n"/>
       <c r="U63" s="10" t="n"/>
+      <c r="V63" s="10" t="n"/>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="9" t="n">
@@ -2526,6 +2610,7 @@
       <c r="S64" s="10" t="n"/>
       <c r="T64" s="10" t="n"/>
       <c r="U64" s="10" t="n"/>
+      <c r="V64" s="10" t="n"/>
     </row>
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="9" t="n">
@@ -2551,6 +2636,7 @@
       <c r="S65" s="10" t="n"/>
       <c r="T65" s="10" t="n"/>
       <c r="U65" s="10" t="n"/>
+      <c r="V65" s="10" t="n"/>
     </row>
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="9" t="n">
@@ -2576,6 +2662,7 @@
       <c r="S66" s="10" t="n"/>
       <c r="T66" s="10" t="n"/>
       <c r="U66" s="10" t="n"/>
+      <c r="V66" s="10" t="n"/>
     </row>
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="9" t="n">
@@ -2601,6 +2688,7 @@
       <c r="S67" s="10" t="n"/>
       <c r="T67" s="10" t="n"/>
       <c r="U67" s="10" t="n"/>
+      <c r="V67" s="10" t="n"/>
     </row>
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="9" t="n">
@@ -2626,6 +2714,7 @@
       <c r="S68" s="10" t="n"/>
       <c r="T68" s="10" t="n"/>
       <c r="U68" s="10" t="n"/>
+      <c r="V68" s="10" t="n"/>
     </row>
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="9" t="n">
@@ -2651,6 +2740,7 @@
       <c r="S69" s="10" t="n"/>
       <c r="T69" s="10" t="n"/>
       <c r="U69" s="10" t="n"/>
+      <c r="V69" s="10" t="n"/>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="9" t="n">
@@ -2676,6 +2766,7 @@
       <c r="S70" s="10" t="n"/>
       <c r="T70" s="10" t="n"/>
       <c r="U70" s="10" t="n"/>
+      <c r="V70" s="10" t="n"/>
     </row>
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="9" t="n">
@@ -2701,6 +2792,7 @@
       <c r="S71" s="10" t="n"/>
       <c r="T71" s="10" t="n"/>
       <c r="U71" s="10" t="n"/>
+      <c r="V71" s="10" t="n"/>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="9" t="n">
@@ -2726,6 +2818,7 @@
       <c r="S72" s="10" t="n"/>
       <c r="T72" s="10" t="n"/>
       <c r="U72" s="10" t="n"/>
+      <c r="V72" s="10" t="n"/>
     </row>
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="9" t="n">
@@ -2751,6 +2844,7 @@
       <c r="S73" s="10" t="n"/>
       <c r="T73" s="10" t="n"/>
       <c r="U73" s="10" t="n"/>
+      <c r="V73" s="10" t="n"/>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="9" t="n">
@@ -2776,6 +2870,7 @@
       <c r="S74" s="10" t="n"/>
       <c r="T74" s="10" t="n"/>
       <c r="U74" s="10" t="n"/>
+      <c r="V74" s="10" t="n"/>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="9" t="n">
@@ -2801,6 +2896,7 @@
       <c r="S75" s="10" t="n"/>
       <c r="T75" s="10" t="n"/>
       <c r="U75" s="10" t="n"/>
+      <c r="V75" s="10" t="n"/>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="9" t="n">
@@ -2826,6 +2922,7 @@
       <c r="S76" s="10" t="n"/>
       <c r="T76" s="10" t="n"/>
       <c r="U76" s="10" t="n"/>
+      <c r="V76" s="10" t="n"/>
     </row>
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="9" t="n">
@@ -2851,6 +2948,7 @@
       <c r="S77" s="10" t="n"/>
       <c r="T77" s="10" t="n"/>
       <c r="U77" s="10" t="n"/>
+      <c r="V77" s="10" t="n"/>
     </row>
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="9" t="n">
@@ -2876,6 +2974,7 @@
       <c r="S78" s="10" t="n"/>
       <c r="T78" s="10" t="n"/>
       <c r="U78" s="10" t="n"/>
+      <c r="V78" s="10" t="n"/>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="9" t="n">
@@ -2901,6 +3000,7 @@
       <c r="S79" s="10" t="n"/>
       <c r="T79" s="10" t="n"/>
       <c r="U79" s="10" t="n"/>
+      <c r="V79" s="10" t="n"/>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="9" t="n">
@@ -2926,6 +3026,7 @@
       <c r="S80" s="10" t="n"/>
       <c r="T80" s="10" t="n"/>
       <c r="U80" s="10" t="n"/>
+      <c r="V80" s="10" t="n"/>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="9" t="n">
@@ -2951,6 +3052,7 @@
       <c r="S81" s="10" t="n"/>
       <c r="T81" s="10" t="n"/>
       <c r="U81" s="10" t="n"/>
+      <c r="V81" s="10" t="n"/>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="9" t="n">
@@ -2976,6 +3078,7 @@
       <c r="S82" s="10" t="n"/>
       <c r="T82" s="10" t="n"/>
       <c r="U82" s="10" t="n"/>
+      <c r="V82" s="10" t="n"/>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="9" t="n">
@@ -3001,6 +3104,7 @@
       <c r="S83" s="10" t="n"/>
       <c r="T83" s="10" t="n"/>
       <c r="U83" s="10" t="n"/>
+      <c r="V83" s="10" t="n"/>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="9" t="n">
@@ -3026,6 +3130,7 @@
       <c r="S84" s="10" t="n"/>
       <c r="T84" s="10" t="n"/>
       <c r="U84" s="10" t="n"/>
+      <c r="V84" s="10" t="n"/>
     </row>
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="9" t="n">
@@ -3051,6 +3156,7 @@
       <c r="S85" s="10" t="n"/>
       <c r="T85" s="10" t="n"/>
       <c r="U85" s="10" t="n"/>
+      <c r="V85" s="10" t="n"/>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="9" t="n">
@@ -3076,6 +3182,7 @@
       <c r="S86" s="10" t="n"/>
       <c r="T86" s="10" t="n"/>
       <c r="U86" s="10" t="n"/>
+      <c r="V86" s="10" t="n"/>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="9" t="n">
@@ -3101,6 +3208,7 @@
       <c r="S87" s="10" t="n"/>
       <c r="T87" s="10" t="n"/>
       <c r="U87" s="10" t="n"/>
+      <c r="V87" s="10" t="n"/>
     </row>
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="9" t="n">
@@ -3126,6 +3234,7 @@
       <c r="S88" s="10" t="n"/>
       <c r="T88" s="10" t="n"/>
       <c r="U88" s="10" t="n"/>
+      <c r="V88" s="10" t="n"/>
     </row>
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="9" t="n">
@@ -3151,6 +3260,7 @@
       <c r="S89" s="10" t="n"/>
       <c r="T89" s="10" t="n"/>
       <c r="U89" s="10" t="n"/>
+      <c r="V89" s="10" t="n"/>
     </row>
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="9" t="n">
@@ -3176,6 +3286,7 @@
       <c r="S90" s="10" t="n"/>
       <c r="T90" s="10" t="n"/>
       <c r="U90" s="10" t="n"/>
+      <c r="V90" s="10" t="n"/>
     </row>
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="9" t="n">
@@ -3201,6 +3312,7 @@
       <c r="S91" s="10" t="n"/>
       <c r="T91" s="10" t="n"/>
       <c r="U91" s="10" t="n"/>
+      <c r="V91" s="10" t="n"/>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="9" t="n">
@@ -3226,6 +3338,7 @@
       <c r="S92" s="10" t="n"/>
       <c r="T92" s="10" t="n"/>
       <c r="U92" s="10" t="n"/>
+      <c r="V92" s="10" t="n"/>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="9" t="n">
@@ -3251,6 +3364,7 @@
       <c r="S93" s="10" t="n"/>
       <c r="T93" s="10" t="n"/>
       <c r="U93" s="10" t="n"/>
+      <c r="V93" s="10" t="n"/>
     </row>
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="9" t="n">
@@ -3276,6 +3390,7 @@
       <c r="S94" s="10" t="n"/>
       <c r="T94" s="10" t="n"/>
       <c r="U94" s="10" t="n"/>
+      <c r="V94" s="10" t="n"/>
     </row>
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="9" t="n">
@@ -3301,6 +3416,7 @@
       <c r="S95" s="10" t="n"/>
       <c r="T95" s="10" t="n"/>
       <c r="U95" s="10" t="n"/>
+      <c r="V95" s="10" t="n"/>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="9" t="n">
@@ -3326,6 +3442,7 @@
       <c r="S96" s="10" t="n"/>
       <c r="T96" s="10" t="n"/>
       <c r="U96" s="10" t="n"/>
+      <c r="V96" s="10" t="n"/>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="9" t="n">
@@ -3351,6 +3468,7 @@
       <c r="S97" s="10" t="n"/>
       <c r="T97" s="10" t="n"/>
       <c r="U97" s="10" t="n"/>
+      <c r="V97" s="10" t="n"/>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="9" t="n">
@@ -3376,6 +3494,7 @@
       <c r="S98" s="10" t="n"/>
       <c r="T98" s="10" t="n"/>
       <c r="U98" s="10" t="n"/>
+      <c r="V98" s="10" t="n"/>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="9" t="n">
@@ -3401,6 +3520,7 @@
       <c r="S99" s="10" t="n"/>
       <c r="T99" s="10" t="n"/>
       <c r="U99" s="10" t="n"/>
+      <c r="V99" s="10" t="n"/>
     </row>
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="9" t="n">
@@ -3426,6 +3546,7 @@
       <c r="S100" s="10" t="n"/>
       <c r="T100" s="10" t="n"/>
       <c r="U100" s="10" t="n"/>
+      <c r="V100" s="10" t="n"/>
     </row>
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="9" t="n">
@@ -3451,6 +3572,7 @@
       <c r="S101" s="10" t="n"/>
       <c r="T101" s="10" t="n"/>
       <c r="U101" s="10" t="n"/>
+      <c r="V101" s="10" t="n"/>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="9" t="n">
@@ -3476,6 +3598,7 @@
       <c r="S102" s="10" t="n"/>
       <c r="T102" s="10" t="n"/>
       <c r="U102" s="10" t="n"/>
+      <c r="V102" s="10" t="n"/>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="9" t="n">
@@ -3501,6 +3624,7 @@
       <c r="S103" s="10" t="n"/>
       <c r="T103" s="10" t="n"/>
       <c r="U103" s="10" t="n"/>
+      <c r="V103" s="10" t="n"/>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="9" t="n">
@@ -3526,6 +3650,7 @@
       <c r="S104" s="10" t="n"/>
       <c r="T104" s="10" t="n"/>
       <c r="U104" s="10" t="n"/>
+      <c r="V104" s="10" t="n"/>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="9" t="n">
@@ -3551,6 +3676,7 @@
       <c r="S105" s="10" t="n"/>
       <c r="T105" s="10" t="n"/>
       <c r="U105" s="10" t="n"/>
+      <c r="V105" s="10" t="n"/>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="9" t="n">
@@ -3576,6 +3702,7 @@
       <c r="S106" s="10" t="n"/>
       <c r="T106" s="10" t="n"/>
       <c r="U106" s="10" t="n"/>
+      <c r="V106" s="10" t="n"/>
     </row>
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="9" t="n">
@@ -3601,6 +3728,7 @@
       <c r="S107" s="10" t="n"/>
       <c r="T107" s="10" t="n"/>
       <c r="U107" s="10" t="n"/>
+      <c r="V107" s="10" t="n"/>
     </row>
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="9" t="n">
@@ -3626,6 +3754,7 @@
       <c r="S108" s="10" t="n"/>
       <c r="T108" s="10" t="n"/>
       <c r="U108" s="10" t="n"/>
+      <c r="V108" s="10" t="n"/>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="9" t="n">
@@ -3651,6 +3780,7 @@
       <c r="S109" s="10" t="n"/>
       <c r="T109" s="10" t="n"/>
       <c r="U109" s="10" t="n"/>
+      <c r="V109" s="10" t="n"/>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="9" t="n">
@@ -3676,6 +3806,7 @@
       <c r="S110" s="10" t="n"/>
       <c r="T110" s="10" t="n"/>
       <c r="U110" s="10" t="n"/>
+      <c r="V110" s="10" t="n"/>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="9" t="n">
@@ -3701,6 +3832,7 @@
       <c r="S111" s="10" t="n"/>
       <c r="T111" s="10" t="n"/>
       <c r="U111" s="10" t="n"/>
+      <c r="V111" s="10" t="n"/>
     </row>
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="9" t="n">
@@ -3726,6 +3858,7 @@
       <c r="S112" s="10" t="n"/>
       <c r="T112" s="10" t="n"/>
       <c r="U112" s="10" t="n"/>
+      <c r="V112" s="10" t="n"/>
     </row>
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="9" t="n">
@@ -3751,6 +3884,7 @@
       <c r="S113" s="10" t="n"/>
       <c r="T113" s="10" t="n"/>
       <c r="U113" s="10" t="n"/>
+      <c r="V113" s="10" t="n"/>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="9" t="n">
@@ -3776,6 +3910,7 @@
       <c r="S114" s="10" t="n"/>
       <c r="T114" s="10" t="n"/>
       <c r="U114" s="10" t="n"/>
+      <c r="V114" s="10" t="n"/>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="9" t="n">
@@ -3801,6 +3936,7 @@
       <c r="S115" s="10" t="n"/>
       <c r="T115" s="10" t="n"/>
       <c r="U115" s="10" t="n"/>
+      <c r="V115" s="10" t="n"/>
     </row>
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="9" t="n">
@@ -3826,6 +3962,7 @@
       <c r="S116" s="10" t="n"/>
       <c r="T116" s="10" t="n"/>
       <c r="U116" s="10" t="n"/>
+      <c r="V116" s="10" t="n"/>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="9" t="n">
@@ -3851,6 +3988,7 @@
       <c r="S117" s="10" t="n"/>
       <c r="T117" s="10" t="n"/>
       <c r="U117" s="10" t="n"/>
+      <c r="V117" s="10" t="n"/>
     </row>
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="9" t="n">
@@ -3876,6 +4014,7 @@
       <c r="S118" s="10" t="n"/>
       <c r="T118" s="10" t="n"/>
       <c r="U118" s="10" t="n"/>
+      <c r="V118" s="10" t="n"/>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="9" t="n">
@@ -3901,6 +4040,7 @@
       <c r="S119" s="10" t="n"/>
       <c r="T119" s="10" t="n"/>
       <c r="U119" s="10" t="n"/>
+      <c r="V119" s="10" t="n"/>
     </row>
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="9" t="n">
@@ -3926,6 +4066,7 @@
       <c r="S120" s="10" t="n"/>
       <c r="T120" s="10" t="n"/>
       <c r="U120" s="10" t="n"/>
+      <c r="V120" s="10" t="n"/>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="9" t="n">
@@ -3951,6 +4092,7 @@
       <c r="S121" s="10" t="n"/>
       <c r="T121" s="10" t="n"/>
       <c r="U121" s="10" t="n"/>
+      <c r="V121" s="10" t="n"/>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="9" t="n">
@@ -3976,6 +4118,7 @@
       <c r="S122" s="10" t="n"/>
       <c r="T122" s="10" t="n"/>
       <c r="U122" s="10" t="n"/>
+      <c r="V122" s="10" t="n"/>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="9" t="n">
@@ -4001,6 +4144,7 @@
       <c r="S123" s="10" t="n"/>
       <c r="T123" s="10" t="n"/>
       <c r="U123" s="10" t="n"/>
+      <c r="V123" s="10" t="n"/>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="9" t="n">
@@ -4026,6 +4170,7 @@
       <c r="S124" s="10" t="n"/>
       <c r="T124" s="10" t="n"/>
       <c r="U124" s="10" t="n"/>
+      <c r="V124" s="10" t="n"/>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="9" t="n">
@@ -4051,6 +4196,7 @@
       <c r="S125" s="10" t="n"/>
       <c r="T125" s="10" t="n"/>
       <c r="U125" s="10" t="n"/>
+      <c r="V125" s="10" t="n"/>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="9" t="n">
@@ -4076,6 +4222,7 @@
       <c r="S126" s="10" t="n"/>
       <c r="T126" s="10" t="n"/>
       <c r="U126" s="10" t="n"/>
+      <c r="V126" s="10" t="n"/>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="9" t="n">
@@ -4101,6 +4248,7 @@
       <c r="S127" s="10" t="n"/>
       <c r="T127" s="10" t="n"/>
       <c r="U127" s="10" t="n"/>
+      <c r="V127" s="10" t="n"/>
     </row>
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="9" t="n">
@@ -4126,6 +4274,7 @@
       <c r="S128" s="10" t="n"/>
       <c r="T128" s="10" t="n"/>
       <c r="U128" s="10" t="n"/>
+      <c r="V128" s="10" t="n"/>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="9" t="n">
@@ -4151,6 +4300,7 @@
       <c r="S129" s="10" t="n"/>
       <c r="T129" s="10" t="n"/>
       <c r="U129" s="10" t="n"/>
+      <c r="V129" s="10" t="n"/>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="9" t="n">
@@ -4176,6 +4326,7 @@
       <c r="S130" s="10" t="n"/>
       <c r="T130" s="10" t="n"/>
       <c r="U130" s="10" t="n"/>
+      <c r="V130" s="10" t="n"/>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="9" t="n">
@@ -4201,6 +4352,7 @@
       <c r="S131" s="10" t="n"/>
       <c r="T131" s="10" t="n"/>
       <c r="U131" s="10" t="n"/>
+      <c r="V131" s="10" t="n"/>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="9" t="n">
@@ -4226,6 +4378,7 @@
       <c r="S132" s="10" t="n"/>
       <c r="T132" s="10" t="n"/>
       <c r="U132" s="10" t="n"/>
+      <c r="V132" s="10" t="n"/>
     </row>
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="9" t="n">
@@ -4251,6 +4404,7 @@
       <c r="S133" s="10" t="n"/>
       <c r="T133" s="10" t="n"/>
       <c r="U133" s="10" t="n"/>
+      <c r="V133" s="10" t="n"/>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="9" t="n">
@@ -4276,6 +4430,7 @@
       <c r="S134" s="10" t="n"/>
       <c r="T134" s="10" t="n"/>
       <c r="U134" s="10" t="n"/>
+      <c r="V134" s="10" t="n"/>
     </row>
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="9" t="n">
@@ -4301,6 +4456,7 @@
       <c r="S135" s="10" t="n"/>
       <c r="T135" s="10" t="n"/>
       <c r="U135" s="10" t="n"/>
+      <c r="V135" s="10" t="n"/>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="9" t="n">
@@ -4326,6 +4482,7 @@
       <c r="S136" s="10" t="n"/>
       <c r="T136" s="10" t="n"/>
       <c r="U136" s="10" t="n"/>
+      <c r="V136" s="10" t="n"/>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="9" t="n">
@@ -4351,6 +4508,7 @@
       <c r="S137" s="10" t="n"/>
       <c r="T137" s="10" t="n"/>
       <c r="U137" s="10" t="n"/>
+      <c r="V137" s="10" t="n"/>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="9" t="n">
@@ -4376,6 +4534,7 @@
       <c r="S138" s="10" t="n"/>
       <c r="T138" s="10" t="n"/>
       <c r="U138" s="10" t="n"/>
+      <c r="V138" s="10" t="n"/>
     </row>
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="9" t="n">
@@ -4401,6 +4560,7 @@
       <c r="S139" s="10" t="n"/>
       <c r="T139" s="10" t="n"/>
       <c r="U139" s="10" t="n"/>
+      <c r="V139" s="10" t="n"/>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="9" t="n">
@@ -4426,6 +4586,7 @@
       <c r="S140" s="10" t="n"/>
       <c r="T140" s="10" t="n"/>
       <c r="U140" s="10" t="n"/>
+      <c r="V140" s="10" t="n"/>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="9" t="n">
@@ -4451,6 +4612,7 @@
       <c r="S141" s="10" t="n"/>
       <c r="T141" s="10" t="n"/>
       <c r="U141" s="10" t="n"/>
+      <c r="V141" s="10" t="n"/>
     </row>
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="9" t="n">
@@ -4476,6 +4638,7 @@
       <c r="S142" s="10" t="n"/>
       <c r="T142" s="10" t="n"/>
       <c r="U142" s="10" t="n"/>
+      <c r="V142" s="10" t="n"/>
     </row>
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="9" t="n">
@@ -4501,6 +4664,7 @@
       <c r="S143" s="10" t="n"/>
       <c r="T143" s="10" t="n"/>
       <c r="U143" s="10" t="n"/>
+      <c r="V143" s="10" t="n"/>
     </row>
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="9" t="n">
@@ -4526,6 +4690,7 @@
       <c r="S144" s="10" t="n"/>
       <c r="T144" s="10" t="n"/>
       <c r="U144" s="10" t="n"/>
+      <c r="V144" s="10" t="n"/>
     </row>
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="9" t="n">
@@ -4551,6 +4716,7 @@
       <c r="S145" s="10" t="n"/>
       <c r="T145" s="10" t="n"/>
       <c r="U145" s="10" t="n"/>
+      <c r="V145" s="10" t="n"/>
     </row>
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="9" t="n">
@@ -4576,6 +4742,7 @@
       <c r="S146" s="10" t="n"/>
       <c r="T146" s="10" t="n"/>
       <c r="U146" s="10" t="n"/>
+      <c r="V146" s="10" t="n"/>
     </row>
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="9" t="n">
@@ -4601,6 +4768,7 @@
       <c r="S147" s="10" t="n"/>
       <c r="T147" s="10" t="n"/>
       <c r="U147" s="10" t="n"/>
+      <c r="V147" s="10" t="n"/>
     </row>
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="9" t="n">
@@ -4626,6 +4794,7 @@
       <c r="S148" s="10" t="n"/>
       <c r="T148" s="10" t="n"/>
       <c r="U148" s="10" t="n"/>
+      <c r="V148" s="10" t="n"/>
     </row>
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="9" t="n">
@@ -4651,6 +4820,7 @@
       <c r="S149" s="10" t="n"/>
       <c r="T149" s="10" t="n"/>
       <c r="U149" s="10" t="n"/>
+      <c r="V149" s="10" t="n"/>
     </row>
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="9" t="n">
@@ -4676,6 +4846,7 @@
       <c r="S150" s="10" t="n"/>
       <c r="T150" s="10" t="n"/>
       <c r="U150" s="10" t="n"/>
+      <c r="V150" s="10" t="n"/>
     </row>
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="9" t="n">
@@ -4701,6 +4872,7 @@
       <c r="S151" s="10" t="n"/>
       <c r="T151" s="10" t="n"/>
       <c r="U151" s="10" t="n"/>
+      <c r="V151" s="10" t="n"/>
     </row>
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="9" t="n">
@@ -4726,6 +4898,7 @@
       <c r="S152" s="10" t="n"/>
       <c r="T152" s="10" t="n"/>
       <c r="U152" s="10" t="n"/>
+      <c r="V152" s="10" t="n"/>
     </row>
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="9" t="n">
@@ -4751,6 +4924,7 @@
       <c r="S153" s="10" t="n"/>
       <c r="T153" s="10" t="n"/>
       <c r="U153" s="10" t="n"/>
+      <c r="V153" s="10" t="n"/>
     </row>
     <row r="154" ht="16" customHeight="1">
       <c r="A154" s="9" t="n">
@@ -4776,6 +4950,7 @@
       <c r="S154" s="10" t="n"/>
       <c r="T154" s="10" t="n"/>
       <c r="U154" s="10" t="n"/>
+      <c r="V154" s="10" t="n"/>
     </row>
     <row r="155" ht="16" customHeight="1">
       <c r="A155" s="9" t="n">
@@ -4801,6 +4976,7 @@
       <c r="S155" s="10" t="n"/>
       <c r="T155" s="10" t="n"/>
       <c r="U155" s="10" t="n"/>
+      <c r="V155" s="10" t="n"/>
     </row>
     <row r="156" ht="16" customHeight="1">
       <c r="A156" s="9" t="n">
@@ -4826,6 +5002,7 @@
       <c r="S156" s="10" t="n"/>
       <c r="T156" s="10" t="n"/>
       <c r="U156" s="10" t="n"/>
+      <c r="V156" s="10" t="n"/>
     </row>
     <row r="157" ht="16" customHeight="1">
       <c r="A157" s="9" t="n">
@@ -4851,6 +5028,7 @@
       <c r="S157" s="10" t="n"/>
       <c r="T157" s="10" t="n"/>
       <c r="U157" s="10" t="n"/>
+      <c r="V157" s="10" t="n"/>
     </row>
     <row r="158" ht="16" customHeight="1">
       <c r="A158" s="9" t="n">
@@ -4876,6 +5054,7 @@
       <c r="S158" s="10" t="n"/>
       <c r="T158" s="10" t="n"/>
       <c r="U158" s="10" t="n"/>
+      <c r="V158" s="10" t="n"/>
     </row>
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="9" t="n">
@@ -4901,6 +5080,7 @@
       <c r="S159" s="10" t="n"/>
       <c r="T159" s="10" t="n"/>
       <c r="U159" s="10" t="n"/>
+      <c r="V159" s="10" t="n"/>
     </row>
     <row r="160" ht="16" customHeight="1">
       <c r="A160" s="9" t="n">
@@ -4926,6 +5106,7 @@
       <c r="S160" s="10" t="n"/>
       <c r="T160" s="10" t="n"/>
       <c r="U160" s="10" t="n"/>
+      <c r="V160" s="10" t="n"/>
     </row>
     <row r="161" ht="16" customHeight="1">
       <c r="A161" s="9" t="n">
@@ -4951,6 +5132,7 @@
       <c r="S161" s="10" t="n"/>
       <c r="T161" s="10" t="n"/>
       <c r="U161" s="10" t="n"/>
+      <c r="V161" s="10" t="n"/>
     </row>
     <row r="162" ht="16" customHeight="1">
       <c r="A162" s="9" t="n">
@@ -4976,6 +5158,7 @@
       <c r="S162" s="10" t="n"/>
       <c r="T162" s="10" t="n"/>
       <c r="U162" s="10" t="n"/>
+      <c r="V162" s="10" t="n"/>
     </row>
     <row r="163" ht="16" customHeight="1">
       <c r="A163" s="9" t="n">
@@ -5001,6 +5184,7 @@
       <c r="S163" s="10" t="n"/>
       <c r="T163" s="10" t="n"/>
       <c r="U163" s="10" t="n"/>
+      <c r="V163" s="10" t="n"/>
     </row>
     <row r="164" ht="16" customHeight="1">
       <c r="A164" s="9" t="n">
@@ -5026,6 +5210,7 @@
       <c r="S164" s="10" t="n"/>
       <c r="T164" s="10" t="n"/>
       <c r="U164" s="10" t="n"/>
+      <c r="V164" s="10" t="n"/>
     </row>
     <row r="165" ht="16" customHeight="1">
       <c r="A165" s="9" t="n">
@@ -5051,6 +5236,7 @@
       <c r="S165" s="10" t="n"/>
       <c r="T165" s="10" t="n"/>
       <c r="U165" s="10" t="n"/>
+      <c r="V165" s="10" t="n"/>
     </row>
     <row r="166" ht="16" customHeight="1">
       <c r="A166" s="9" t="n">
@@ -5076,6 +5262,7 @@
       <c r="S166" s="10" t="n"/>
       <c r="T166" s="10" t="n"/>
       <c r="U166" s="10" t="n"/>
+      <c r="V166" s="10" t="n"/>
     </row>
     <row r="167" ht="16" customHeight="1">
       <c r="A167" s="9" t="n">
@@ -5101,6 +5288,7 @@
       <c r="S167" s="10" t="n"/>
       <c r="T167" s="10" t="n"/>
       <c r="U167" s="10" t="n"/>
+      <c r="V167" s="10" t="n"/>
     </row>
     <row r="168" ht="16" customHeight="1">
       <c r="A168" s="9" t="n">
@@ -5126,6 +5314,7 @@
       <c r="S168" s="10" t="n"/>
       <c r="T168" s="10" t="n"/>
       <c r="U168" s="10" t="n"/>
+      <c r="V168" s="10" t="n"/>
     </row>
     <row r="169" ht="16" customHeight="1">
       <c r="A169" s="9" t="n">
@@ -5151,6 +5340,7 @@
       <c r="S169" s="10" t="n"/>
       <c r="T169" s="10" t="n"/>
       <c r="U169" s="10" t="n"/>
+      <c r="V169" s="10" t="n"/>
     </row>
     <row r="170" ht="16" customHeight="1">
       <c r="A170" s="9" t="n">
@@ -5176,6 +5366,7 @@
       <c r="S170" s="10" t="n"/>
       <c r="T170" s="10" t="n"/>
       <c r="U170" s="10" t="n"/>
+      <c r="V170" s="10" t="n"/>
     </row>
     <row r="171" ht="16" customHeight="1">
       <c r="A171" s="9" t="n">
@@ -5201,6 +5392,7 @@
       <c r="S171" s="10" t="n"/>
       <c r="T171" s="10" t="n"/>
       <c r="U171" s="10" t="n"/>
+      <c r="V171" s="10" t="n"/>
     </row>
     <row r="172" ht="16" customHeight="1">
       <c r="A172" s="9" t="n">
@@ -5226,6 +5418,7 @@
       <c r="S172" s="10" t="n"/>
       <c r="T172" s="10" t="n"/>
       <c r="U172" s="10" t="n"/>
+      <c r="V172" s="10" t="n"/>
     </row>
     <row r="173" ht="16" customHeight="1">
       <c r="A173" s="9" t="n">
@@ -5251,6 +5444,7 @@
       <c r="S173" s="10" t="n"/>
       <c r="T173" s="10" t="n"/>
       <c r="U173" s="10" t="n"/>
+      <c r="V173" s="10" t="n"/>
     </row>
     <row r="174" ht="16" customHeight="1">
       <c r="A174" s="9" t="n">
@@ -5276,6 +5470,7 @@
       <c r="S174" s="10" t="n"/>
       <c r="T174" s="10" t="n"/>
       <c r="U174" s="10" t="n"/>
+      <c r="V174" s="10" t="n"/>
     </row>
     <row r="175" ht="16" customHeight="1">
       <c r="A175" s="9" t="n">
@@ -5301,6 +5496,7 @@
       <c r="S175" s="10" t="n"/>
       <c r="T175" s="10" t="n"/>
       <c r="U175" s="10" t="n"/>
+      <c r="V175" s="10" t="n"/>
     </row>
     <row r="176" ht="16" customHeight="1">
       <c r="A176" s="9" t="n">
@@ -5326,6 +5522,7 @@
       <c r="S176" s="10" t="n"/>
       <c r="T176" s="10" t="n"/>
       <c r="U176" s="10" t="n"/>
+      <c r="V176" s="10" t="n"/>
     </row>
     <row r="177" ht="16" customHeight="1">
       <c r="A177" s="9" t="n">
@@ -5351,6 +5548,7 @@
       <c r="S177" s="10" t="n"/>
       <c r="T177" s="10" t="n"/>
       <c r="U177" s="10" t="n"/>
+      <c r="V177" s="10" t="n"/>
     </row>
     <row r="178" ht="16" customHeight="1">
       <c r="A178" s="9" t="n">
@@ -5376,6 +5574,7 @@
       <c r="S178" s="10" t="n"/>
       <c r="T178" s="10" t="n"/>
       <c r="U178" s="10" t="n"/>
+      <c r="V178" s="10" t="n"/>
     </row>
     <row r="179" ht="16" customHeight="1">
       <c r="A179" s="9" t="n">
@@ -5401,6 +5600,7 @@
       <c r="S179" s="10" t="n"/>
       <c r="T179" s="10" t="n"/>
       <c r="U179" s="10" t="n"/>
+      <c r="V179" s="10" t="n"/>
     </row>
     <row r="180" ht="16" customHeight="1">
       <c r="A180" s="9" t="n">
@@ -5426,6 +5626,7 @@
       <c r="S180" s="10" t="n"/>
       <c r="T180" s="10" t="n"/>
       <c r="U180" s="10" t="n"/>
+      <c r="V180" s="10" t="n"/>
     </row>
     <row r="181" ht="16" customHeight="1">
       <c r="A181" s="9" t="n">
@@ -5451,6 +5652,7 @@
       <c r="S181" s="10" t="n"/>
       <c r="T181" s="10" t="n"/>
       <c r="U181" s="10" t="n"/>
+      <c r="V181" s="10" t="n"/>
     </row>
     <row r="182" ht="16" customHeight="1">
       <c r="A182" s="9" t="n">
@@ -5476,6 +5678,7 @@
       <c r="S182" s="10" t="n"/>
       <c r="T182" s="10" t="n"/>
       <c r="U182" s="10" t="n"/>
+      <c r="V182" s="10" t="n"/>
     </row>
     <row r="183" ht="16" customHeight="1">
       <c r="A183" s="9" t="n">
@@ -5501,6 +5704,7 @@
       <c r="S183" s="10" t="n"/>
       <c r="T183" s="10" t="n"/>
       <c r="U183" s="10" t="n"/>
+      <c r="V183" s="10" t="n"/>
     </row>
     <row r="184" ht="16" customHeight="1">
       <c r="A184" s="9" t="n">
@@ -5526,6 +5730,7 @@
       <c r="S184" s="10" t="n"/>
       <c r="T184" s="10" t="n"/>
       <c r="U184" s="10" t="n"/>
+      <c r="V184" s="10" t="n"/>
     </row>
     <row r="185" ht="16" customHeight="1">
       <c r="A185" s="9" t="n">
@@ -5551,6 +5756,7 @@
       <c r="S185" s="10" t="n"/>
       <c r="T185" s="10" t="n"/>
       <c r="U185" s="10" t="n"/>
+      <c r="V185" s="10" t="n"/>
     </row>
     <row r="186" ht="16" customHeight="1">
       <c r="A186" s="9" t="n">
@@ -5576,6 +5782,7 @@
       <c r="S186" s="10" t="n"/>
       <c r="T186" s="10" t="n"/>
       <c r="U186" s="10" t="n"/>
+      <c r="V186" s="10" t="n"/>
     </row>
     <row r="187" ht="16" customHeight="1">
       <c r="A187" s="9" t="n">
@@ -5601,6 +5808,7 @@
       <c r="S187" s="10" t="n"/>
       <c r="T187" s="10" t="n"/>
       <c r="U187" s="10" t="n"/>
+      <c r="V187" s="10" t="n"/>
     </row>
     <row r="188" ht="16" customHeight="1">
       <c r="A188" s="9" t="n">
@@ -5626,6 +5834,7 @@
       <c r="S188" s="10" t="n"/>
       <c r="T188" s="10" t="n"/>
       <c r="U188" s="10" t="n"/>
+      <c r="V188" s="10" t="n"/>
     </row>
     <row r="189" ht="16" customHeight="1">
       <c r="A189" s="9" t="n">
@@ -5651,6 +5860,7 @@
       <c r="S189" s="10" t="n"/>
       <c r="T189" s="10" t="n"/>
       <c r="U189" s="10" t="n"/>
+      <c r="V189" s="10" t="n"/>
     </row>
     <row r="190" ht="16" customHeight="1">
       <c r="A190" s="9" t="n">
@@ -5676,6 +5886,7 @@
       <c r="S190" s="10" t="n"/>
       <c r="T190" s="10" t="n"/>
       <c r="U190" s="10" t="n"/>
+      <c r="V190" s="10" t="n"/>
     </row>
     <row r="191" ht="16" customHeight="1">
       <c r="A191" s="9" t="n">
@@ -5701,6 +5912,7 @@
       <c r="S191" s="10" t="n"/>
       <c r="T191" s="10" t="n"/>
       <c r="U191" s="10" t="n"/>
+      <c r="V191" s="10" t="n"/>
     </row>
     <row r="192" ht="16" customHeight="1">
       <c r="A192" s="9" t="n">
@@ -5726,6 +5938,7 @@
       <c r="S192" s="10" t="n"/>
       <c r="T192" s="10" t="n"/>
       <c r="U192" s="10" t="n"/>
+      <c r="V192" s="10" t="n"/>
     </row>
     <row r="193" ht="16" customHeight="1">
       <c r="A193" s="9" t="n">
@@ -5751,6 +5964,7 @@
       <c r="S193" s="10" t="n"/>
       <c r="T193" s="10" t="n"/>
       <c r="U193" s="10" t="n"/>
+      <c r="V193" s="10" t="n"/>
     </row>
     <row r="194" ht="16" customHeight="1">
       <c r="A194" s="9" t="n">
@@ -5776,6 +5990,7 @@
       <c r="S194" s="10" t="n"/>
       <c r="T194" s="10" t="n"/>
       <c r="U194" s="10" t="n"/>
+      <c r="V194" s="10" t="n"/>
     </row>
     <row r="195" ht="16" customHeight="1">
       <c r="A195" s="9" t="n">
@@ -5801,6 +6016,7 @@
       <c r="S195" s="10" t="n"/>
       <c r="T195" s="10" t="n"/>
       <c r="U195" s="10" t="n"/>
+      <c r="V195" s="10" t="n"/>
     </row>
     <row r="196" ht="16" customHeight="1">
       <c r="A196" s="9" t="n">
@@ -5826,6 +6042,7 @@
       <c r="S196" s="10" t="n"/>
       <c r="T196" s="10" t="n"/>
       <c r="U196" s="10" t="n"/>
+      <c r="V196" s="10" t="n"/>
     </row>
     <row r="197" ht="16" customHeight="1">
       <c r="A197" s="9" t="n">
@@ -5851,6 +6068,7 @@
       <c r="S197" s="10" t="n"/>
       <c r="T197" s="10" t="n"/>
       <c r="U197" s="10" t="n"/>
+      <c r="V197" s="10" t="n"/>
     </row>
     <row r="198" ht="16" customHeight="1">
       <c r="A198" s="9" t="n">
@@ -5876,6 +6094,7 @@
       <c r="S198" s="10" t="n"/>
       <c r="T198" s="10" t="n"/>
       <c r="U198" s="10" t="n"/>
+      <c r="V198" s="10" t="n"/>
     </row>
     <row r="199" ht="16" customHeight="1">
       <c r="A199" s="9" t="n">
@@ -5901,6 +6120,7 @@
       <c r="S199" s="10" t="n"/>
       <c r="T199" s="10" t="n"/>
       <c r="U199" s="10" t="n"/>
+      <c r="V199" s="10" t="n"/>
     </row>
     <row r="200" ht="16" customHeight="1">
       <c r="A200" s="9" t="n">
@@ -5926,6 +6146,7 @@
       <c r="S200" s="10" t="n"/>
       <c r="T200" s="10" t="n"/>
       <c r="U200" s="10" t="n"/>
+      <c r="V200" s="10" t="n"/>
     </row>
     <row r="201" ht="16" customHeight="1">
       <c r="A201" s="9" t="n">
@@ -5951,6 +6172,7 @@
       <c r="S201" s="10" t="n"/>
       <c r="T201" s="10" t="n"/>
       <c r="U201" s="10" t="n"/>
+      <c r="V201" s="10" t="n"/>
     </row>
     <row r="202" ht="16" customHeight="1">
       <c r="A202" s="9" t="n">
@@ -5976,6 +6198,7 @@
       <c r="S202" s="10" t="n"/>
       <c r="T202" s="10" t="n"/>
       <c r="U202" s="10" t="n"/>
+      <c r="V202" s="10" t="n"/>
     </row>
     <row r="203" ht="16" customHeight="1">
       <c r="A203" s="9" t="n">
@@ -6001,26 +6224,30 @@
       <c r="S203" s="10" t="n"/>
       <c r="T203" s="10" t="n"/>
       <c r="U203" s="10" t="n"/>
+      <c r="V203" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="J1:L1"/>
-    <mergeCell ref="M1:R1"/>
-    <mergeCell ref="S1:U1"/>
+    <mergeCell ref="T1:V1"/>
+    <mergeCell ref="M1:S1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation sqref="F4:F203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Gender" prompt="Select gender" type="list">
       <formula1>"Male,Female,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="R4:R203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Employee Status" prompt="Select status" type="list">
       <formula1>"Active,Inactive,Suspended"</formula1>
     </dataValidation>
-    <dataValidation sqref="T4:T203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Skill Level" prompt="Select skill level" type="list">
+    <dataValidation sqref="U4:U203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Skill Level" prompt="Select skill level" type="list">
       <formula1>"Beginner,Intermediate,Advanced"</formula1>
     </dataValidation>
-    <dataValidation sqref="U4:U203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Training Needed" prompt="Yes or No" type="list">
+    <dataValidation sqref="V4:V203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Training Needed" prompt="Yes or No" type="list">
       <formula1>"Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="S4:S203" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" promptTitle="Access Level" prompt="Select system access level" type="list">
+      <formula1>"Administrator,Management,Human Resources,Head of Department,Employee"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>